<commit_message>
Enrutamiento red viñedo 1
</commit_message>
<xml_diff>
--- a/VLSM Automatico.xlsx
+++ b/VLSM Automatico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Redes y protocolos de comunicación\Trabajo_Final\Redes_Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0C4FB6-7AE3-44FD-B9D1-B25C8A8D67C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{315A1DBB-DC6A-4F19-A508-CC3BAD66F011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1020" yWindow="1488" windowWidth="12792" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="91">
   <si>
     <t>Estructura de Planificación de Red VLSM</t>
   </si>
@@ -162,13 +162,157 @@
   </si>
   <si>
     <t>Campo viñedo 3</t>
+  </si>
+  <si>
+    <t>VIÑEDO 1</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Router_Viñedo_1</t>
+  </si>
+  <si>
+    <t>PC_Viñedo_1</t>
+  </si>
+  <si>
+    <t>192.168.10.1</t>
+  </si>
+  <si>
+    <t>192.168.10.2</t>
+  </si>
+  <si>
+    <t>Router_Campo_1</t>
+  </si>
+  <si>
+    <t>192.168.10.17</t>
+  </si>
+  <si>
+    <t>192.168.10.18</t>
+  </si>
+  <si>
+    <t>192.168.10.19</t>
+  </si>
+  <si>
+    <t>192.168.10.20</t>
+  </si>
+  <si>
+    <t>192.168.10.21</t>
+  </si>
+  <si>
+    <t>192.168.10.22</t>
+  </si>
+  <si>
+    <t>MCU_Norte_1</t>
+  </si>
+  <si>
+    <t>Tablet_Viñedo_1</t>
+  </si>
+  <si>
+    <t>192.168.10.3</t>
+  </si>
+  <si>
+    <t>255.255.255.248</t>
+  </si>
+  <si>
+    <t>VIÑEDO 2</t>
+  </si>
+  <si>
+    <t>VIÑEDO 3</t>
+  </si>
+  <si>
+    <t>Router_Viñedo_2</t>
+  </si>
+  <si>
+    <t>PC_Viñedo_2</t>
+  </si>
+  <si>
+    <t>Tablet_Viñedo_2</t>
+  </si>
+  <si>
+    <t>Router_Viñedo_3</t>
+  </si>
+  <si>
+    <t>PC_Viñedo_3</t>
+  </si>
+  <si>
+    <t>Tablet_Viñedo_3</t>
+  </si>
+  <si>
+    <t>Router_Campo_2</t>
+  </si>
+  <si>
+    <t>MCU_Norte_2</t>
+  </si>
+  <si>
+    <t>MCU_Oeste_1</t>
+  </si>
+  <si>
+    <t>MCU_Sur_1</t>
+  </si>
+  <si>
+    <t>MCU_Este_1</t>
+  </si>
+  <si>
+    <t>MCU_Oeste_2</t>
+  </si>
+  <si>
+    <t>MCU_Sur_2</t>
+  </si>
+  <si>
+    <t>MCU_Este_2</t>
+  </si>
+  <si>
+    <t>Router_Campo_3</t>
+  </si>
+  <si>
+    <t>MCU_Norte_3</t>
+  </si>
+  <si>
+    <t>MCU_Oeste_3</t>
+  </si>
+  <si>
+    <t>MCU_Sur_3</t>
+  </si>
+  <si>
+    <t>MCU_Este_3</t>
+  </si>
+  <si>
+    <t>192.168.10.33</t>
+  </si>
+  <si>
+    <t>192.168.10.34</t>
+  </si>
+  <si>
+    <t>192.168.10.35</t>
+  </si>
+  <si>
+    <t>192.168.10.65</t>
+  </si>
+  <si>
+    <t>192.168.10.66</t>
+  </si>
+  <si>
+    <t>192.168.10.67</t>
+  </si>
+  <si>
+    <t>255.255.255.240</t>
+  </si>
+  <si>
+    <t>Laptop_Campo_1</t>
+  </si>
+  <si>
+    <t>Laptop_Campo_2</t>
+  </si>
+  <si>
+    <t>Laptop_Campo_3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -188,8 +332,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -202,8 +354,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -226,18 +396,97 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -266,7 +515,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>841617</xdr:colOff>
+      <xdr:colOff>841616</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>148593</xdr:rowOff>
     </xdr:to>
@@ -505,7 +754,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
@@ -513,10 +762,11 @@
     <col min="3" max="3" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" customWidth="1"/>
     <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.109375" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1353,7 +1603,7 @@
       </c>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1489,7 +1739,7 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+      <c r="A32" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1625,11 +1875,340 @@
       </c>
     </row>
     <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
+      <c r="A39" t="s">
         <v>39</v>
       </c>
     </row>
+    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="17"/>
+      <c r="E41" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F41" s="13"/>
+      <c r="G41" s="14"/>
+      <c r="I41" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J41" s="13"/>
+      <c r="K41" s="14"/>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="10"/>
+      <c r="C42" s="11"/>
+      <c r="E42" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="10"/>
+      <c r="G42" s="11"/>
+      <c r="I42" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J42" s="10"/>
+      <c r="K42" s="11"/>
+    </row>
+    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="K45" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="10"/>
+      <c r="C46" s="11"/>
+      <c r="E46" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F46" s="10"/>
+      <c r="G46" s="11"/>
+      <c r="I46" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="J46" s="10"/>
+      <c r="K46" s="11"/>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G57" s="8"/>
+    </row>
+    <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G60" s="8"/>
+    </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="E42:G42"/>
+    <mergeCell ref="E46:G46"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Conexión a router general
- Corrección de la segmentación de redes
- Enrutamiento de viñedos hacia router central
</commit_message>
<xml_diff>
--- a/VLSM Automatico.xlsx
+++ b/VLSM Automatico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Redes y protocolos de comunicación\Trabajo_Final\Redes_Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FBC5499-BB53-4B82-A0D5-27FB7BD32B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA00EC64-0054-4182-975C-E5A1AF08FFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14292" yWindow="0" windowWidth="8844" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14280" yWindow="0" windowWidth="8856" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="137">
   <si>
     <t>Ubicación / Nombre de Red</t>
   </si>
@@ -429,6 +429,21 @@
   </si>
   <si>
     <t>Router_Oficina</t>
+  </si>
+  <si>
+    <t>192.168.100.24</t>
+  </si>
+  <si>
+    <t>192.168.100.25</t>
+  </si>
+  <si>
+    <t>192.168.100.26</t>
+  </si>
+  <si>
+    <t>192.168.100.27</t>
+  </si>
+  <si>
+    <t>Router_Google</t>
   </si>
 </sst>
 </file>
@@ -596,16 +611,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -617,20 +632,24 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -898,7 +917,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A3:M83"/>
+  <dimension ref="A3:M79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.109375" customWidth="1"/>
@@ -924,9 +943,9 @@
       <c r="C3" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -938,9 +957,9 @@
       <c r="C4" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -952,9 +971,9 @@
       <c r="C5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -966,9 +985,9 @@
       <c r="C6" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -980,9 +999,9 @@
       <c r="C7" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -994,9 +1013,9 @@
       <c r="C8" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -1008,27 +1027,26 @@
       <c r="C9" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
+      <c r="A11" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1157,14 +1175,14 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="23" t="s">
+      <c r="A17" t="s">
         <v>77</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1907,55 +1925,41 @@
       </c>
     </row>
     <row r="51" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="23"/>
-      <c r="B51" s="23"/>
-      <c r="C51" s="23"/>
-      <c r="D51" s="23"/>
-      <c r="E51" s="23"/>
-      <c r="F51" s="23"/>
-      <c r="G51" s="23"/>
-      <c r="H51" s="23"/>
-      <c r="I51" s="23"/>
-      <c r="J51" s="23"/>
-      <c r="K51" s="23"/>
-      <c r="L51" s="23"/>
       <c r="M51" s="7"/>
     </row>
     <row r="52" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="13" t="s">
+      <c r="A52" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="14"/>
-      <c r="C52" s="15"/>
-      <c r="E52" s="16" t="s">
+      <c r="B52" s="16"/>
+      <c r="C52" s="17"/>
+      <c r="E52" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F52" s="17"/>
-      <c r="G52" s="18"/>
-      <c r="I52" s="16" t="s">
+      <c r="F52" s="13"/>
+      <c r="G52" s="14"/>
+      <c r="I52" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J52" s="17"/>
-      <c r="K52" s="18"/>
-      <c r="L52" s="23"/>
+      <c r="J52" s="13"/>
+      <c r="K52" s="14"/>
     </row>
     <row r="53" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="12" t="s">
+      <c r="A53" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B53" s="10"/>
-      <c r="C53" s="11"/>
-      <c r="E53" s="12" t="s">
+      <c r="B53" s="19"/>
+      <c r="C53" s="20"/>
+      <c r="E53" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F53" s="10"/>
-      <c r="G53" s="11"/>
-      <c r="I53" s="12" t="s">
+      <c r="F53" s="19"/>
+      <c r="G53" s="20"/>
+      <c r="I53" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="J53" s="10"/>
-      <c r="K53" s="11"/>
-      <c r="L53" s="23"/>
+      <c r="J53" s="19"/>
+      <c r="K53" s="20"/>
     </row>
     <row r="54" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
@@ -1985,7 +1989,6 @@
       <c r="K54" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L54" s="23"/>
     </row>
     <row r="55" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
@@ -2015,7 +2018,6 @@
       <c r="K55" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L55" s="23"/>
     </row>
     <row r="56" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
@@ -2045,25 +2047,23 @@
       <c r="K56" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L56" s="23"/>
     </row>
     <row r="57" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B57" s="10"/>
-      <c r="C57" s="11"/>
-      <c r="E57" s="12" t="s">
+      <c r="B57" s="19"/>
+      <c r="C57" s="20"/>
+      <c r="E57" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="F57" s="10"/>
-      <c r="G57" s="11"/>
-      <c r="I57" s="12" t="s">
+      <c r="F57" s="19"/>
+      <c r="G57" s="20"/>
+      <c r="I57" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="J57" s="10"/>
-      <c r="K57" s="11"/>
-      <c r="L57" s="23"/>
+      <c r="J57" s="19"/>
+      <c r="K57" s="20"/>
     </row>
     <row r="58" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
@@ -2087,13 +2087,12 @@
       <c r="I58" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="J58" s="5" t="s">
+      <c r="J58" s="11" t="s">
         <v>90</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L58" s="23"/>
     </row>
     <row r="59" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
@@ -2123,7 +2122,6 @@
       <c r="K59" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L59" s="23"/>
     </row>
     <row r="60" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
@@ -2153,7 +2151,6 @@
       <c r="K60" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L60" s="23"/>
     </row>
     <row r="61" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
@@ -2183,7 +2180,6 @@
       <c r="K61" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L61" s="23"/>
     </row>
     <row r="62" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
@@ -2213,7 +2209,6 @@
       <c r="K62" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L62" s="23"/>
     </row>
     <row r="63" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
@@ -2243,28 +2238,25 @@
       <c r="K63" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L63" s="23"/>
     </row>
     <row r="64" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="9" t="s">
+      <c r="A64" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B64" s="10"/>
-      <c r="C64" s="11"/>
-      <c r="E64" s="9" t="s">
+      <c r="B64" s="19"/>
+      <c r="C64" s="20"/>
+      <c r="E64" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="F64" s="10"/>
-      <c r="G64" s="11"/>
-      <c r="I64" s="9" t="s">
+      <c r="F64" s="19"/>
+      <c r="G64" s="20"/>
+      <c r="I64" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="J64" s="10"/>
-      <c r="K64" s="11"/>
-      <c r="L64" s="23"/>
-      <c r="M64" s="23"/>
-    </row>
-    <row r="65" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J64" s="19"/>
+      <c r="K64" s="20"/>
+    </row>
+    <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>68</v>
       </c>
@@ -2292,10 +2284,8 @@
       <c r="K65" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L65" s="23"/>
-      <c r="M65" s="23"/>
-    </row>
-    <row r="66" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>32</v>
       </c>
@@ -2323,10 +2313,8 @@
       <c r="K66" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L66" s="23"/>
-      <c r="M66" s="23"/>
-    </row>
-    <row r="67" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>36</v>
       </c>
@@ -2354,10 +2342,8 @@
       <c r="K67" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L67" s="23"/>
-      <c r="M67" s="23"/>
-    </row>
-    <row r="68" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>9</v>
       </c>
@@ -2385,28 +2371,25 @@
       <c r="K68" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="L68" s="23"/>
-      <c r="M68" s="23"/>
-    </row>
-    <row r="69" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="9" t="s">
+    </row>
+    <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B69" s="10"/>
-      <c r="C69" s="11"/>
-      <c r="E69" s="9" t="s">
+      <c r="B69" s="22"/>
+      <c r="C69" s="23"/>
+      <c r="E69" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="F69" s="10"/>
-      <c r="G69" s="11"/>
-      <c r="I69" s="9" t="s">
+      <c r="F69" s="19"/>
+      <c r="G69" s="20"/>
+      <c r="I69" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="J69" s="10"/>
-      <c r="K69" s="11"/>
-      <c r="M69" s="23"/>
-    </row>
-    <row r="70" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J69" s="19"/>
+      <c r="K69" s="20"/>
+    </row>
+    <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>68</v>
       </c>
@@ -2434,11 +2417,10 @@
       <c r="K70" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M70" s="23"/>
-    </row>
-    <row r="71" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>32</v>
+        <v>131</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>106</v>
@@ -2446,8 +2428,8 @@
       <c r="C71" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E71" s="2" t="s">
-        <v>42</v>
+      <c r="E71" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>114</v>
@@ -2455,8 +2437,8 @@
       <c r="G71" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="I71" s="2" t="s">
-        <v>45</v>
+      <c r="I71" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="J71" s="2" t="s">
         <v>122</v>
@@ -2464,11 +2446,10 @@
       <c r="K71" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M71" s="23"/>
-    </row>
-    <row r="72" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="3" t="s">
-        <v>131</v>
+    </row>
+    <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>107</v>
@@ -2476,8 +2457,8 @@
       <c r="C72" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E72" s="3" t="s">
-        <v>131</v>
+      <c r="E72" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>115</v>
@@ -2485,8 +2466,8 @@
       <c r="G72" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="I72" s="3" t="s">
-        <v>131</v>
+      <c r="I72" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="J72" s="2" t="s">
         <v>123</v>
@@ -2494,9 +2475,8 @@
       <c r="K72" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M72" s="23"/>
-    </row>
-    <row r="73" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>9</v>
       </c>
@@ -2524,56 +2504,77 @@
       <c r="K73" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="M73" s="23"/>
-    </row>
-    <row r="74" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M74" s="23"/>
-    </row>
-    <row r="75" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M75" s="23"/>
-    </row>
-    <row r="76" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M76" s="23"/>
-    </row>
-    <row r="77" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B75" s="22"/>
+      <c r="C75" s="23"/>
+    </row>
+    <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="I77" s="8"/>
-      <c r="M77" s="23"/>
-    </row>
-    <row r="78" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M78" s="23"/>
-    </row>
-    <row r="79" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M79" s="23"/>
-    </row>
-    <row r="80" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M80" s="23"/>
-    </row>
-    <row r="81" spans="13:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M81" s="23"/>
-    </row>
-    <row r="82" spans="13:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M82" s="23"/>
-    </row>
-    <row r="83" spans="13:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M83" s="23"/>
+    </row>
+    <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="E69:G69"/>
+    <mergeCell ref="I69:K69"/>
+    <mergeCell ref="A75:C75"/>
+    <mergeCell ref="I57:K57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="I64:K64"/>
     <mergeCell ref="E52:G52"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="E53:G53"/>
     <mergeCell ref="I53:K53"/>
     <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="E57:G57"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="E69:G69"/>
-    <mergeCell ref="I69:K69"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Configuracion de rede y oficina
</commit_message>
<xml_diff>
--- a/VLSM Automatico.xlsx
+++ b/VLSM Automatico.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Redes y protocolos de comunicación\Trabajo_Final\Redes_Final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luciel\Documents\GitHub\Redes_Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA00EC64-0054-4182-975C-E5A1AF08FFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89DC804D-89CC-49C6-8D2A-448331FB2864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14280" yWindow="0" windowWidth="8856" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="140">
   <si>
     <t>Ubicación / Nombre de Red</t>
   </si>
@@ -444,6 +444,15 @@
   </si>
   <si>
     <t>Router_Google</t>
+  </si>
+  <si>
+    <t>RRHH</t>
+  </si>
+  <si>
+    <t>Servidores</t>
+  </si>
+  <si>
+    <t>Google</t>
   </si>
 </sst>
 </file>
@@ -614,6 +623,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -630,24 +657,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -918,22 +927,22 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A3:M79"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.109375" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="17.44140625" customWidth="1"/>
-    <col min="10" max="10" width="16.5546875" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" customWidth="1"/>
+    <col min="10" max="10" width="16.5703125" customWidth="1"/>
     <col min="11" max="11" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -947,7 +956,7 @@
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -961,7 +970,7 @@
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -975,7 +984,7 @@
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -989,7 +998,7 @@
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -1003,7 +1012,7 @@
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1017,7 +1026,7 @@
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
@@ -1031,14 +1040,14 @@
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>76</v>
       </c>
@@ -1048,12 +1057,12 @@
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>0</v>
       </c>
@@ -1088,7 +1097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -1131,7 +1140,7 @@
         <v>255.255.255.224</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1174,7 +1183,7 @@
         <v>255.255.255.224</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -1184,12 +1193,12 @@
       <c r="E17" s="9"/>
       <c r="F17" s="10"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>0</v>
       </c>
@@ -1224,7 +1233,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
@@ -1267,7 +1276,7 @@
         <v>255.255.255.224</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
@@ -1310,12 +1319,12 @@
         <v>255.255.255.224</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>0</v>
       </c>
@@ -1350,7 +1359,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>29</v>
       </c>
@@ -1393,7 +1402,7 @@
         <v>255.255.255.224</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>28</v>
       </c>
@@ -1436,17 +1445,17 @@
         <v>255.255.255.224</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>0</v>
       </c>
@@ -1481,20 +1490,48 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2"/>
+    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>139</v>
+      </c>
       <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
-    </row>
-    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C31" s="1">
+        <v>0</v>
+      </c>
+      <c r="D31" s="1">
+        <f t="array" ref="D31">MATCH(TRUE, (2^{0;1;2;3;4;5;6;7;8}) &gt;= (B31+2), 0) - 1</f>
+        <v>1</v>
+      </c>
+      <c r="E31" s="1">
+        <f>2^D31</f>
+        <v>2</v>
+      </c>
+      <c r="F31" s="1">
+        <f>32-D31</f>
+        <v>31</v>
+      </c>
+      <c r="G31" s="1" t="str">
+        <f>CONCATENATE("192.168.40.",C31)</f>
+        <v>192.168.40.0</v>
+      </c>
+      <c r="H31" s="1" t="str">
+        <f>CONCATENATE("192.168.40.",C31 +1)</f>
+        <v>192.168.40.1</v>
+      </c>
+      <c r="I31" s="1" t="str">
+        <f>CONCATENATE("192.168.40.",C31 + E31 - 2)</f>
+        <v>192.168.40.0</v>
+      </c>
+      <c r="J31" s="1" t="str">
+        <f>CONCATENATE("192.168.40.",C31 + E31 - 1)</f>
+        <v>192.168.40.1</v>
+      </c>
+      <c r="K31" s="1" t="str">
+        <f>CONCATENATE("255.255.255.", 256 - E31)</f>
+        <v>255.255.255.254</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1507,17 +1544,17 @@
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>0</v>
       </c>
@@ -1552,43 +1589,103 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
-    </row>
-    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-    </row>
-    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B37" s="1">
+        <v>20</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0</v>
+      </c>
+      <c r="D37" s="1">
+        <f t="array" ref="D37">MATCH(TRUE, (2^{0;1;2;3;4;5;6;7;8}) &gt;= (B37+2), 0) - 1</f>
+        <v>5</v>
+      </c>
+      <c r="E37" s="1">
+        <f>2^D37</f>
+        <v>32</v>
+      </c>
+      <c r="F37" s="1">
+        <f>32-D37</f>
+        <v>27</v>
+      </c>
+      <c r="G37" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C37)</f>
+        <v>192.168.50.0</v>
+      </c>
+      <c r="H37" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C37 +1)</f>
+        <v>192.168.50.1</v>
+      </c>
+      <c r="I37" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C37 + E37 - 2)</f>
+        <v>192.168.50.30</v>
+      </c>
+      <c r="J37" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C37 + E37 - 1)</f>
+        <v>192.168.50.31</v>
+      </c>
+      <c r="K37" s="1" t="str">
+        <f>CONCATENATE("255.255.255.", 256 - E37)</f>
+        <v>255.255.255.224</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B38" s="1">
+        <v>20</v>
+      </c>
+      <c r="C38" s="1">
+        <v>32</v>
+      </c>
+      <c r="D38" s="1">
+        <f t="array" ref="D38">MATCH(TRUE, (2^{0;1;2;3;4;5;6;7;8}) &gt;= (B38+2), 0) - 1</f>
+        <v>5</v>
+      </c>
+      <c r="E38" s="1">
+        <f>2^D38</f>
+        <v>32</v>
+      </c>
+      <c r="F38" s="1">
+        <f>32-D38</f>
+        <v>27</v>
+      </c>
+      <c r="G38" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C38)</f>
+        <v>192.168.50.32</v>
+      </c>
+      <c r="H38" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C38 +1)</f>
+        <v>192.168.50.33</v>
+      </c>
+      <c r="I38" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C38 + E38 - 2)</f>
+        <v>192.168.50.62</v>
+      </c>
+      <c r="J38" s="1" t="str">
+        <f>CONCATENATE("192.168.50.",C38 + E38 - 1)</f>
+        <v>192.168.50.63</v>
+      </c>
+      <c r="K38" s="1" t="str">
+        <f>CONCATENATE("255.255.255.", 256 - E38)</f>
+        <v>255.255.255.224</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>0</v>
       </c>
@@ -1623,7 +1720,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>16</v>
       </c>
@@ -1666,7 +1763,7 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>84</v>
       </c>
@@ -1709,7 +1806,7 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>18</v>
       </c>
@@ -1752,7 +1849,7 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>19</v>
       </c>
@@ -1795,7 +1892,7 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -1838,7 +1935,7 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>21</v>
       </c>
@@ -1881,7 +1978,7 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>22</v>
       </c>
@@ -1924,44 +2021,44 @@
         <v>255.255.255.252</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M51" s="7"/>
     </row>
-    <row r="52" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="15" t="s">
+    <row r="52" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="16"/>
-      <c r="C52" s="17"/>
-      <c r="E52" s="12" t="s">
+      <c r="B52" s="22"/>
+      <c r="C52" s="23"/>
+      <c r="E52" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="F52" s="13"/>
-      <c r="G52" s="14"/>
-      <c r="I52" s="12" t="s">
+      <c r="F52" s="19"/>
+      <c r="G52" s="20"/>
+      <c r="I52" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="J52" s="13"/>
-      <c r="K52" s="14"/>
-    </row>
-    <row r="53" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="18" t="s">
+      <c r="J52" s="19"/>
+      <c r="K52" s="20"/>
+    </row>
+    <row r="53" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B53" s="19"/>
-      <c r="C53" s="20"/>
-      <c r="E53" s="18" t="s">
+      <c r="B53" s="15"/>
+      <c r="C53" s="16"/>
+      <c r="E53" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F53" s="19"/>
-      <c r="G53" s="20"/>
-      <c r="I53" s="18" t="s">
+      <c r="F53" s="15"/>
+      <c r="G53" s="16"/>
+      <c r="I53" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="J53" s="19"/>
-      <c r="K53" s="20"/>
-    </row>
-    <row r="54" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J53" s="15"/>
+      <c r="K53" s="16"/>
+    </row>
+    <row r="54" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>32</v>
       </c>
@@ -1990,7 +2087,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>33</v>
       </c>
@@ -2019,7 +2116,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>38</v>
       </c>
@@ -2048,24 +2145,24 @@
         <v>80</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="18" t="s">
+    <row r="57" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="B57" s="19"/>
-      <c r="C57" s="20"/>
-      <c r="E57" s="18" t="s">
+      <c r="B57" s="15"/>
+      <c r="C57" s="16"/>
+      <c r="E57" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="F57" s="19"/>
-      <c r="G57" s="20"/>
-      <c r="I57" s="18" t="s">
+      <c r="F57" s="15"/>
+      <c r="G57" s="16"/>
+      <c r="I57" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="J57" s="19"/>
-      <c r="K57" s="20"/>
-    </row>
-    <row r="58" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J57" s="15"/>
+      <c r="K57" s="16"/>
+    </row>
+    <row r="58" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>36</v>
       </c>
@@ -2094,7 +2191,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>37</v>
       </c>
@@ -2123,7 +2220,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>50</v>
       </c>
@@ -2152,7 +2249,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>51</v>
       </c>
@@ -2181,7 +2278,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
         <v>52</v>
       </c>
@@ -2210,7 +2307,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>64</v>
       </c>
@@ -2239,24 +2336,24 @@
         <v>80</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="21" t="s">
+    <row r="64" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B64" s="19"/>
-      <c r="C64" s="20"/>
-      <c r="E64" s="21" t="s">
+      <c r="B64" s="15"/>
+      <c r="C64" s="16"/>
+      <c r="E64" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F64" s="19"/>
-      <c r="G64" s="20"/>
-      <c r="I64" s="21" t="s">
+      <c r="F64" s="15"/>
+      <c r="G64" s="16"/>
+      <c r="I64" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="J64" s="19"/>
-      <c r="K64" s="20"/>
-    </row>
-    <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J64" s="15"/>
+      <c r="K64" s="16"/>
+    </row>
+    <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>68</v>
       </c>
@@ -2285,7 +2382,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>32</v>
       </c>
@@ -2314,7 +2411,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>36</v>
       </c>
@@ -2343,7 +2440,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>9</v>
       </c>
@@ -2372,24 +2469,24 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="21" t="s">
+    <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B69" s="22"/>
-      <c r="C69" s="23"/>
-      <c r="E69" s="21" t="s">
+      <c r="B69" s="13"/>
+      <c r="C69" s="14"/>
+      <c r="E69" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="F69" s="19"/>
-      <c r="G69" s="20"/>
-      <c r="I69" s="21" t="s">
+      <c r="F69" s="15"/>
+      <c r="G69" s="16"/>
+      <c r="I69" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="J69" s="19"/>
-      <c r="K69" s="20"/>
-    </row>
-    <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J69" s="15"/>
+      <c r="K69" s="16"/>
+    </row>
+    <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>68</v>
       </c>
@@ -2418,7 +2515,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>131</v>
       </c>
@@ -2447,7 +2544,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>32</v>
       </c>
@@ -2476,7 +2573,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>9</v>
       </c>
@@ -2505,14 +2602,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="21" t="s">
+    <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B75" s="22"/>
-      <c r="C75" s="23"/>
-    </row>
-    <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="13"/>
+      <c r="C75" s="14"/>
+    </row>
+    <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>68</v>
       </c>
@@ -2523,7 +2620,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>131</v>
       </c>
@@ -2535,7 +2632,7 @@
       </c>
       <c r="I77" s="8"/>
     </row>
-    <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>136</v>
       </c>
@@ -2546,7 +2643,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>9</v>
       </c>
@@ -2559,6 +2656,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="I52:K52"/>
     <mergeCell ref="A69:C69"/>
     <mergeCell ref="E69:G69"/>
     <mergeCell ref="I69:K69"/>
@@ -2569,12 +2672,6 @@
     <mergeCell ref="A64:C64"/>
     <mergeCell ref="E64:G64"/>
     <mergeCell ref="I64:K64"/>
-    <mergeCell ref="E52:G52"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="I52:K52"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>